<commit_message>
Add completeness risk matrix and release 0.1.1
</commit_message>
<xml_diff>
--- a/samples/DCP_clean_v0.1/dataflow_collection_template_v0.1.xlsx
+++ b/samples/DCP_clean_v0.1/dataflow_collection_template_v0.1.xlsx
@@ -3353,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R38"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3424,8 +3424,6 @@
       <c r="Q2" s="1" t="n"/>
       <c r="R2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -3737,7 +3735,7 @@
       </c>
       <c r="I8" s="44" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J8" s="44" t="inlineStr">
@@ -4745,6 +4743,98 @@
       <c r="P38" s="47" t="str"/>
       <c r="Q38" s="63" t="str"/>
       <c r="R38" s="48" t="str"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MON-009</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>mon-da-push</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>svc-da-push</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>metrics+logging+alert</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://grafana.example/d/da-push</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>da-push-delivery-failure</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Covered</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Testnetv2</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>dashboard_link</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>EV-014</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>collector</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Clean sample monitoring coverage for DA push module.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5833,8 +5923,6 @@
       <c r="R2" s="1" t="n"/>
       <c r="S2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -11085,8 +11173,6 @@
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -12295,8 +12381,6 @@
       <c r="T2" s="1" t="n"/>
       <c r="U2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -16405,8 +16489,6 @@
       <c r="V2" s="1" t="n"/>
       <c r="W2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -18923,8 +19005,6 @@
       <c r="W2" s="1" t="n"/>
       <c r="X2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>

</xml_diff>